<commit_message>
Dashboard + reports full check: W2 results and consolidated findings pack
W2 (Sales By Customer/Representative, Sales, Advisor Analysis, Technician Efficiency,
Sales Tax Collected, Follow Up) complete; TAX1 re-verified live by coordinator.
Consolidated report + workbook: 4 ready to file, 16 held for PO, 8 already reported,
4 reopen decisions, 43 PO questions. Nothing filed in Jira, TestRail untouched.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D95Q7VoyGzYXAt4w5J2bJE
</commit_message>
<xml_diff>
--- a/build/dashboard-verify-2026-10-28/ShopView-Dashboard-and-Reports-Full-Check-Findings-2026-10-28.xlsx
+++ b/build/dashboard-verify-2026-10-28/ShopView-Dashboard-and-Reports-Full-Check-Findings-2026-10-28.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
@@ -564,7 +564,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
@@ -767,36 +767,210 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Parts Velocity + Inventory Value</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
+          <t>Parts Velocity</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>2034770</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>2034573</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>197</v>
+      </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>see reports/W3-parts/RESULTS.md — 2 ready-to-file drafts</t>
+          <t>168 = PV-D1; rest explained (deleted parts PQ-6, collation, inconclusive slices); seeded data → PV-D1, PV-D2</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
+          <t>Inventory Value</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>800233</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>800226</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>collation / unrounded ties — invisible on screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
           <t>A/R, A/P, IBS, QB Unexported, Exports, Notes, Reminders</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B23" s="3" t="n">
         <v>824</v>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C23" s="3" t="n">
         <v>756</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D23" s="3" t="n">
         <v>68</v>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>1 ready, 4 held, 2 known</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Sales By Customer</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>144175</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>129838</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>14337</v>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>mostly spec-vs-ticket label/date-basis rows (SQ-1, SQ-4, SQ-10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Sales By Representative</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>147584</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>146093</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>1491</v>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>277 = rep changed after invoicing (correct); SV-8974; SQ-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Sales (remaining columns)</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>97250</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>96171</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>1079</v>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>every failure matches the invoice record (Stats tab changed later)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Service Advisor Analysis</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>113291</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>112690</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>601</v>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>as Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Technician Efficiency (both tabs)</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1089952</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>1089118</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>834</v>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>F2 declined lines (101); tiny clocks (SQ-6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Sales Tax Collected (2 passes) + void + filters</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>582213</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>563613</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>18074</v>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>TAX1 ready; pass-1 status failures replaced by pass 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Follow Up (hidden)</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>server error every read (SQ-5)</t>
         </is>
       </c>
     </row>
@@ -811,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1013,6 +1187,53 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>TAX1</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Sales Tax Collected</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>An invoice part-paid by a deposit shows Invoice Status "Paid", and the "Partially Paid" filter leaves it out.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Reproduced twice (S1-38212; S1-38214 made fully through the screen) + 9 older invoices in 2 other locations. Coordinator re-read live 28 Oct: S1-38214 own record partially_paid, open balance $105.00; Sales Tax row "paid"; Partially Paid filter returns 0 rows. Sales By Representative shows it partially paid.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>SV-4573 (Done): "Invoice Status (, Partially Paid, Paid)" — quote re-read live by coordinator</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>reports/W2-sales-advisor-tax/defects/TICKET-W2-6-sales-tax-status-deposit-paid.wiki</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/defects/TICKET-W2-6-sales-tax-status-deposit-paid.wiki</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1024,7 +1245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1508,6 +1729,335 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>SBC1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Sales By Customer</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Margin % divides by Subtotal minus Shop Supplies; the SBC and SBR specs disagree on the base.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>6,464 rows.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>SBC spec Confluence 577634305 v22 (2026-10-19) vs SBR spec 585629698 v30 §3</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>SQ-1</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>reports/W2-sales-advisor-tax/defects/TICKET-W2-1-sbc-margin-percent-base.wiki</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/defects/TICKET-W2-1-sbc-margin-percent-base.wiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>DEC1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>SBC / SBR / Sales</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Labor Delta and Margin % show 2 decimals (specs say 1); negative money shows "(-$2.50)".</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Every row.</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>SBC v22 / SBR v30</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>SQ-2</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-labor-delta-and-margin-decimals.md</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-labor-delta-and-margin-decimals.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>SBR2</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Sales By Representative</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>A $0.00 invoice nobody paid shows "Paid".</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>645 invoices.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>SV-9217 vs SBR spec v30 §3</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>SQ-3</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>reports/W2-sales-advisor-tax/RESULTS.md</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/RESULTS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>FU1</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Follow Up (hidden page)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>The hidden Follow Up page is blank and its data request fails (server error) on 12 of 12 reads.</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>12/12 reads HTTP 500.</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>No written source</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>SQ-5</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>reports/W2-sales-advisor-tax/defects/TICKET-W2-5-follow-up-report-server-error.wiki</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/defects/TICKET-W2-5-follow-up-report-server-error.wiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>TE1</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Technician Efficiency</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>A clock shorter than 0.01 h drops the line's whole technician time.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>727 rows, 221 lines.</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>see candidate</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>SQ-6</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-te-tiny-clock-drops-tech-time.md</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-te-tiny-clock-drops-tech-time.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>DATE1</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>SBC / SBR date options</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>The date options on screen match neither spec.</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Screen.</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>SBC v22 / SBR v30</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>SQ-7</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-date-filter-options.md</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-date-filter-options.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>TAX2</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Sales Tax Collected</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Unpaid invoices are not listed; credit-memo tax handling; $0.00 invoices listed "Paid" with no payment (643); deposit invoices dated by invoice not deposit (20).</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>See RESULTS §6.</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>SV-4573</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>SQ-8, SQ-9, SQ-11</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>reports/W2-sales-advisor-tax/RESULTS.md</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/RESULTS.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1519,7 +2069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1909,6 +2459,53 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>SALES-K1</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Margin shows "N/A" when parts are $0.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Screen.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>SV-6147 (open)</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>reports/W2-sales-advisor-tax/RESULTS.md</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/RESULTS.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1920,7 +2517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2122,6 +2719,53 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>SBR1</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Sales By Representative</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Invoices on the same day are not ordered by invoice number.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>8 checks; reproduced on screen twice.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>SV-8974 (closed OBSOLETE 9 Aug 2026 without a fix)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Reopen?</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-sbr-same-day-invoice-order.md</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-sbr-same-day-invoice-order.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2133,7 +2777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2288,6 +2932,100 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>SBC2</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Sales By Customer</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Asset label follows SV-9459, not spec S8-R7; SBC/SBR differ from today's Stats tab after later clocks or credits.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>7,293 / 558 rows. Spec update (SQ-4) and design question (SQ-10).</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>SBC v22, SV-9459</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>SQ-4, SQ-10</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>reports/W2-sales-advisor-tax/RESULTS.md</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/RESULTS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>O4-W2</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Outside reports</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Customer payment window</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Void invoice S1-38207 still shows $135.00 owing in New Customer Payment; work order stays "Invoiced".</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>The invoice was voided through the API only (no screen path) — passed to the payments owner as an observation.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>reports/W2-sales-advisor-tax/RESULTS.md</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/RESULTS.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2299,7 +3037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2653,7 +3391,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>RQ-1</t>
+          <t>SQ-1</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2681,7 +3419,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>RQ-2</t>
+          <t>SQ-2</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2696,12 +3434,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>SBC S12-R2 and SBR S9-R2 say Labor Delta is *"rounded to one decimal"*; SBC S7-R11 says Margin % *"to one decimal"*. SV-9199 / SV-9200 (your tickets, Aug 12) repeat *"signed one-decimal format (+2.0 / -14.0 / 0.0)"*. But SV-9068 and SV-9069 (Done, Aug 10, "SV standard is 2") changed SBC to two decimals, and the build shows two decimals on SBC and SBR (+112.64, +1.00, 82.81 %).</t>
+          <t>SBC S12-R2 and SBR S9-R2 say Labor Delta is *"rounded to one decimal"*; SBC S7-R11 says Margin % *"to one decimal"*. SV-9199 / SV-9200 (your tickets, Aug 12) repeat *"signed one-decimal format (+2.0 / -14.0 / 0.0)"*. But SV-9068 and SV-9069 (Done, Aug 10, "SV standard is 2") changed SBC to two decimals, and the build shows two decimals on SBC and SBR (+112.64, +1.00, 82.81 %). Also: SBR §3 says *"Negative dollar values use accounting-convention parentheses — `($1,234.56)`"*; the SBR screen shows a negative margin as (-$2.50), with both brackets and a minus sign.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Ticket needed (one decimal) / Working as intended — please update S12-R2, S9-R2, S7-R11 to two decimals</t>
+          <t>Ticket needed (one decimal; brackets without the minus sign) / Working as intended — please update S12-R2, S9-R2, S7-R11 to two decimals and the §3 negative-money example</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr"/>
@@ -2709,7 +3447,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>RQ-3</t>
+          <t>SQ-3</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2737,7 +3475,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>RQ-4</t>
+          <t>SQ-4</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2765,7 +3503,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>RQ-5</t>
+          <t>SQ-5</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -2793,7 +3531,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>RQ-6</t>
+          <t>SQ-6</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -2821,7 +3559,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>RQ-7</t>
+          <t>SQ-7</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -2849,7 +3587,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>RQ-8</t>
+          <t>SQ-8</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -2877,7 +3615,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>RQ-9</t>
+          <t>SQ-9</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -2887,17 +3625,17 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Should the tax-rate totals be reduced by tax on credit memos?</t>
+          <t>Should the tax-rate totals take off the tax on credit memos (returns) made in the same dates?</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Not stated anywhere. The backend works out a reduced figure that no screen shows (code note).</t>
+          <t>No document says. Today the screen's footer and the All tax rates tab add up the listed invoices only (checked: they match, 64 of 64 date ranges); credit memos never appear on this report. The server also works out a second, reduced tax total that no screen shows.</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>— / —</t>
+          <t>Ticket needed (show credit memo tax) / Working as intended</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr"/>
@@ -2905,55 +3643,63 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>PQ-1</t>
+          <t>SQ-10</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Report Suite · Parts Velocity</t>
+          <t>Reports · Sales By Customer and Sales By Representative · Labor Delta, Labor Margin, Parts Margin</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Should Last 90 days cover exactly 90 days (today and the 89 days before it)? *Yes / No*</t>
+          <t>When time is clocked, or a cost changes, after an invoice is made, should these reports keep the figures from when the invoice was made?</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Today it covers 91 days: on 28 Oct it runs 30 Jul – 28 Oct. SV-11514 only says "The default range is Last 90 Days."</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr"/>
+          <t>Neither spec says which moment counts. SBC: *"Labor Delta — Hours invoiced minus hours worked"*; SBR §3: *"hours worked = the technician clocked (timesheet) hours recorded against that work order"*, *"Labor Margin = Labor Invoiced − the shop's labor cost"*. On most invoices the reports match the work order's Stats tab exactly. They differ on 370 invoices for Labor Delta, 119 for Labor Margin and 69 for Parts Margin (of about 8,000). All of these are invoices where time was clocked, or parts were credited, after the invoice was made (mostly automated-test customer TestVT1). Example: S2-38022, report Labor Delta +1.00, Stats tab today 2.00 invoiced − 0.00 worked.</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Working as intended — please add "as at the time of invoicing" to both specs / Ticket needed (use today's clocked hours and costs)</t>
+        </is>
+      </c>
       <c r="F22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>PQ-2</t>
+          <t>SQ-11</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Report Suite · Parts Velocity</t>
+          <t>Reports · Sales Tax Collected · Invoice Status and Invoice Paid Date</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Should Revenue, Margin, Avg Cost, Avg Sell, Sold (WO), Sold (Parts Sale) and every Special Order figure be dated by the invoice date? *Yes / No*</t>
+          <t>(a) Should a $0.00 invoice with no payment be listed as "Paid", with a paid date? (b) When a deposit taken before invoicing pays part of an invoice, should Invoice Paid Date be the deposit's date?</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>The spec (Story 5, "Work-order date") dates them by the work order's end date, but work orders do not get an end date (it is empty on the paid work order S2-17193 we opened, and the build's own notes say it is never filled), so the report uses the invoice date. A "Yes" means the spec should be updated; a "No" means we need a different date.</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr"/>
+          <t>(a) 643 $0.00 invoices are listed as Paid with a paid date (the invoice's creation time), but no payment exists. 428 of them read *unpaid* on their own record. This is the same question as SQ-3, for this report. (b) SV-4573: *"for partially paid invoices, show the date of the latest payment"*. On 20 deposit invoices the report shows the time the invoice was made, not the deposit date (e.g. P2-2445: deposit 21 Oct, report 22 Oct). *(Separate from this: the same deposit invoices show "Paid" instead of "Partially Paid". That one is clear from SV-4573 and is drafted as a ticket, `defects/TICKET-W2-6-sales-tax-status-deposit-paid.wiki`.)*</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>(a) Working as intended (b) Ticket needed / (a) Ticket needed (b) Working as intended — please note in the story that a deposit counts on the day it is applied</t>
+        </is>
+      </c>
       <c r="F23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>PQ-3</t>
+          <t>PQ-1</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -2963,12 +3709,12 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Should a return to the vendor made from Parts → Returns count in Units Returned? *Yes / No*</t>
+          <t>Should Last 90 days cover exactly 90 days (today and the 89 days before it)? *Yes / No*</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>It does today (we returned 1 unit of ZZAUTOTEST-PV1-10282011 to the vendor and Units Returned went from 0 to 1; cancelling it put it back to 0). The spec names only "a work-order part return or a parts-sale credit".</t>
+          <t>Today it covers 91 days: on 28 Oct it runs 30 Jul – 28 Oct. SV-11514 only says "The default range is Last 90 Days."</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr"/>
@@ -2977,7 +3723,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>PQ-4</t>
+          <t>PQ-2</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -2987,12 +3733,12 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>When a user who has several locations picks one location, should the Location column be hidden? *Yes / No*</t>
+          <t>Should Revenue, Margin, Avg Cost, Avg Sell, Sold (WO), Sold (Parts Sale) and every Special Order figure be dated by the invoice date? *Yes / No*</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>It is hidden today. The spec says both: S2-R12 "when a single location is in scope the column is hidden", and S3-R10 / Key Decisions "shown by default … regardless of how many locations are currently selected". (This is the same open point as the contested SV-8938.) Inventory Value shows the column with one location selected.</t>
+          <t>The spec (Story 5, "Work-order date") dates them by the work order's end date, but work orders do not get an end date (it is empty on the paid work order S2-17193 we opened, and the build's own notes say it is never filled), so the report uses the invoice date. A "Yes" means the spec should be updated; a "No" means we need a different date.</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr"/>
@@ -3001,7 +3747,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>PQ-5</t>
+          <t>PQ-3</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -3011,12 +3757,12 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Is the date list on screen the intended one — This week, Last week, This month, Last month, This quarter, Last quarter, This year, Last year, Last 90 days, Last 12 months, Custom (no Today, no Yesterday)? *Yes / No*</t>
+          <t>Should a return to the vendor made from Parts → Returns count in Units Returned? *Yes / No*</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>That is what the screen offers, in line with your 5 Aug answer and SV-11514. The spec text (S2-R2) still lists Today and Yesterday and does not list Last 12 months, so a "Yes" means S2-R2 should be updated. Every option's dates were checked and are right.</t>
+          <t>It does today (we returned 1 unit of ZZAUTOTEST-PV1-10282011 to the vendor and Units Returned went from 0 to 1; cancelling it put it back to 0). The spec names only "a work-order part return or a parts-sale credit".</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr"/>
@@ -3025,7 +3771,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>PQ-6</t>
+          <t>PQ-4</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -3035,12 +3781,12 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Should a part's past sales stay in Parts Velocity after the part record is deleted? *Yes / No*</t>
+          <t>When a user who has several locations picks one location, should the Location column be hidden? *Yes / No*</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Today they disappear. Last Year at Staging Heavy Duty - 9919 is missing $2,357.74 of billed sales across 9 parts that no longer exist (for example 84-4005PK, billed on S2-4699, S2-4987, S2-6540). S3-N1 says "A part with billed Revenue &gt; 0 is always kept". We could not delete a sold part from the screen, so we have not raised a ticket.</t>
+          <t>It is hidden today. The spec says both: S2-R12 "when a single location is in scope the column is hidden", and S3-R10 / Key Decisions "shown by default … regardless of how many locations are currently selected". (This is the same open point as the contested SV-8938.) Inventory Value shows the column with one location selected.</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
@@ -3049,7 +3795,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>PQ-7</t>
+          <t>PQ-5</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -3059,12 +3805,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Should Last Sale for a stocked part include a sale that was billed but recorded no stock movement? *Yes / No*</t>
+          <t>Is the date list on screen the intended one — This week, Last week, This month, Last month, This quarter, Last quarter, This year, Last year, Last 90 days, Last 12 months, Custom (no Today, no Yesterday)? *Yes / No*</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Example: N000000001069 at Staging Heavy Duty - 9919 was billed on S2-16621 (30 Jul 2026) but Last Sale reads 160 days (its previous stock-moving sale). S3-N1 calls a billed sale without stock movement "a drop-ship sale"; Last Sale is "the part's most recent sale".</t>
+          <t>That is what the screen offers, in line with your 5 Aug answer and SV-11514. The spec text (S2-R2) still lists Today and Yesterday and does not list Last 12 months, so a "Yes" means S2-R2 should be updated. Every option's dates were checked and are right.</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr"/>
@@ -3073,22 +3819,22 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>PQ-8</t>
+          <t>PQ-6</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Report Suite · Inventory Value</t>
+          <t>Report Suite · Parts Velocity</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>When a part's cost is above the highest price band of its category's pricing matrix, should Unit Sell use that highest band's markup? *Yes / No*</t>
+          <t>Should a part's past sales stay in Parts Velocity after the part record is deleted? *Yes / No*</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>That is what it does today, and it matches the parts list (example: 2599273C92 at Staging Lethbridge - 4310, cost $526.70, category HD-Filters whose bands stop at $500 → Unit Sell $752.44 = +42.86%). The spec only says "the shop's pricing-matrix markup on cost for that part's category".</t>
+          <t>Today they disappear. Last Year at Staging Heavy Duty - 9919 is missing $2,357.74 of billed sales across 9 parts that no longer exist (for example 84-4005PK, billed on S2-4699, S2-4987, S2-6540). S3-N1 says "A part with billed Revenue &gt; 0 is always kept". We could not delete a sold part from the screen, so we have not raised a ticket.</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr"/>
@@ -3097,83 +3843,75 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>RQ-1</t>
+          <t>PQ-7</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>A/R Aging Collection (and A/P Aging Detail) · Past Due</t>
+          <t>Report Suite · Parts Velocity</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Should a credit created ON the chosen date count as 0 days old — so it is left off A/R Aging Collection (and shows Past Due 0 on A/P Aging Detail)?</t>
+          <t>Should Last Sale for a stocked part include a sale that was billed but recorded no stock movement? *Yes / No*</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>The PRD says "If the calculated days are ≤ 0 … it's not shown on the report". Ticket SV-5606 (Done, Jan 2026) asked instead for "Today's Credits … displayed with 1 as a Past Due", and the build does that. Example: CM2-4462 (E2E Credits Customer) created 30 Sep 2026 is listed as 1 day past due on 30 Sep 2026.</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>We file TICKET-AR1 / Working as intended — the PRD wording should be updated to match SV-5606</t>
-        </is>
-      </c>
+          <t>Example: N000000001069 at Staging Heavy Duty - 9919 was billed on S2-16621 (30 Jul 2026) but Last Sale reads 160 days (its previous stock-moving sale). S3-N1 calls a billed sale without stock movement "a drop-ship sale"; Last Sale is "the part's most recent sale".</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr"/>
       <c r="F30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>RQ-2</t>
+          <t>PQ-8</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>A/R Aging · part-sale deposits</t>
+          <t>Report Suite · Inventory Value</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Should a deposit taken on a part sale reduce that part sale's open balance on A/R Aging once the part sale is invoiced (as it already does on the customer's Invoices tab)?</t>
+          <t>When a part's cost is above the highest price band of its category's pricing matrix, should Unit Sell use that highest band's markup? *Yes / No*</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>P2-2352 (TestVT1): Invoices tab $443.43, A/R Aging $543.43 — the $100 deposit DEP-4763 stays "Held" and A/R now leaves held deposits out (SV-11690 fix). Same for P2-2439 ($5).</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>We add this to SV-11690 (comment), or file it on your say-so / Working as intended</t>
-        </is>
-      </c>
+          <t>That is what it does today, and it matches the parts list (example: 2599273C92 at Staging Lethbridge - 4310, cost $526.70, category HD-Filters whose bands stop at $500 → Unit Sell $752.44 = +42.86%). The spec only says "the shop's pricing-matrix markup on cost for that part's category".</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>RQ-3</t>
+          <t>RQ-1</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>IBS Batches · Sent tab</t>
+          <t>A/R Aging Collection (and A/P Aging Detail) · Past Due</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Must a Sent batch's Total always equal the sum of the invoices (and credits) inside it?</t>
+          <t>Should a credit created ON the chosen date count as 0 days old — so it is left off A/R Aging Collection (and shows Past Due 0 on A/P Aging Detail)?</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Lethbridge batch of 2 Oct 2026 shows $9,473.35; its 9 invoices add up to $9,183.29 (its own IBS export also says $9,183.29). We could not find the cause.</t>
+          <t>The PRD says "If the calculated days are ≤ 0 … it's not shown on the report". Ticket SV-5606 (Done, Jan 2026) asked instead for "Today's Credits … displayed with 1 as a Past Due", and the build does that. Example: CM2-4462 (E2E Credits Customer) created 30 Sep 2026 is listed as 1 day past due on 30 Sep 2026.</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>We file TICKET-IBS1 and a developer finds the cause / —</t>
+          <t>We file TICKET-AR1 / Working as intended — the PRD wording should be updated to match SV-5606</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr"/>
@@ -3181,27 +3919,27 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>RQ-4</t>
+          <t>RQ-2</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Notes Report</t>
+          <t>A/R Aging · part-sale deposits</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Should the Notes Report let the user see every note in the chosen range (today it stops at 100)?</t>
+          <t>Should a deposit taken on a part sale reduce that part sale's open balance on A/R Aging once the part sale is invoiced (as it already does on the customer's Invoices tab)?</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>"All" shows 100 of 2,545 notes; "Last Week" 100 of 255; "Filter by Author" 100 of 1,105. There is no "load more". No written spec exists for this report.</t>
+          <t>P2-2352 (TestVT1): Invoices tab $443.43, A/R Aging $543.43 — the $100 deposit DEP-4763 stays "Held" and A/R now leaves held deposits out (SV-11690 fix). Same for P2-2439 ($5).</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>We file TICKET-NOTES1 / Working as intended (the 100 limit should then be stated on screen)</t>
+          <t>We add this to SV-11690 (comment), or file it on your say-so / Working as intended</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr"/>
@@ -3209,27 +3947,27 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>RQ-5</t>
+          <t>RQ-3</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>IBS Batches · Ready to Send</t>
+          <t>IBS Batches · Sent tab</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Should a $0.00 invoice be listed in Ready to Send?</t>
+          <t>Must a Sent batch's Total always equal the sum of the invoices (and credits) inside it?</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>S2-16924 (Fort Mohave Diesel Repair) is listed with Total $0.00 / Balance $0.00, waiting to be sent to IBS.</t>
+          <t>Lethbridge batch of 2 Oct 2026 shows $9,473.35; its 9 invoices add up to $9,183.29 (its own IBS export also says $9,183.29). We could not find the cause.</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>— / We raise it</t>
+          <t>We file TICKET-IBS1 and a developer finds the cause / —</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr"/>
@@ -3237,27 +3975,27 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>RQ-6</t>
+          <t>RQ-4</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>QB Unexported · Customers tab</t>
+          <t>Notes Report</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Should every credit memo row show its credit number (e.g. CM2-4476) in the No. column?</t>
+          <t>Should the Notes Report let the user see every note in the chosen range (today it stops at 100)?</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>All 283 credit-memo rows (Heavy Duty 255, Lethbridge 28) have a blank No.; payments / applications are blank too. 111 documents appear twice with two different errors. No written spec exists for this screen.</t>
+          <t>"All" shows 100 of 2,545 notes; "Last Week" 100 of 255; "Filter by Author" 100 of 1,105. There is no "load more". No written spec exists for this report.</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>We raise it / —</t>
+          <t>We file TICKET-NOTES1 / Working as intended (the 100 limit should then be stated on screen)</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr"/>
@@ -3265,27 +4003,27 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>RQ-7</t>
+          <t>RQ-5</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Export Reports · Customer Invoice</t>
+          <t>IBS Batches · Ready to Send</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Should the Terms column show the invoice's own term?</t>
+          <t>Should a $0.00 invoice be listed in Ready to Send?</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>7 invoices from Sep 2026 show "Net 30/50/60" while the invoice and its customer both say COD and the due date equals the invoice date (e.g. S2-31597).</t>
+          <t>S2-16924 (Fort Mohave Diesel Repair) is listed with Total $0.00 / Balance $0.00, waiting to be sent to IBS.</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>We raise it / —</t>
+          <t>— / We raise it</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr"/>
@@ -3293,27 +4031,27 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>RQ-8</t>
+          <t>RQ-6</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Export Reports · Payroll Timesheet</t>
+          <t>QB Unexported · Customers tab</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Can an employee's day legitimately exceed 24 Total Hours?</t>
+          <t>Should every credit memo row show its credit number (e.g. CM2-4476) in the No. column?</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Sep 2026: Admin Shopview 40.70 h on 10 Sep, 32.34 h on 17 Sep; Haley Brown 28.50 h on 6 Sep (WO Hours from overlapping clocks).</t>
+          <t>All 283 credit-memo rows (Heavy Duty 255, Lethbridge 28) have a blank No.; payments / applications are blank too. 111 documents appear twice with two different errors. No written spec exists for this screen.</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>— / We raise it (also check SV-10701)</t>
+          <t>We raise it / —</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr"/>
@@ -3321,27 +4059,27 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>RQ-9</t>
+          <t>RQ-7</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Export Reports · dates</t>
+          <t>Export Reports · Customer Invoice</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Should the export's dates use the location's own time zone?</t>
+          <t>Should the Terms column show the invoice's own term?</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>For Staging Heavy Duty - 9919 (time zone Asia/Karachi on staging) the Customer Invoice export prints dates one day earlier than the location's calendar date for invoices made late in the UTC day (e.g. S2-31625: 02 Sep in the file, 03 Sep at the location). Lethbridge (Edmonton) matches. Likely only a staging set-up artefact.</t>
+          <t>7 invoices from Sep 2026 show "Net 30/50/60" while the invoice and its customer both say COD and the due date equals the invoice date (e.g. S2-31597).</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>— / —</t>
+          <t>We raise it / —</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr"/>
@@ -3349,27 +4087,27 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>DQ-1</t>
+          <t>RQ-8</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Dashboard · Technician Efficiency (and the Technician Efficiency report)</t>
+          <t>Export Reports · Payroll Timesheet</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>When a customer declines a line, should that line's technician time still count in "Invoiced Tech Hrs" (and its clocked time in "Clocked")?</t>
+          <t>Can an employee's day legitimately exceed 24 Total Hours?</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Today it does. Example S1-38198: only line 1 was billed, yet the technician shows 2.00 Invoiced Tech Hrs and 133.33 %. The Billing Efficiency tile leaves the same declined line out. The PRD calls the figure "invoiced technician hours" but defines it as "technician time *recorded* on work order lines".</t>
+          <t>Sep 2026: Admin Shopview 40.70 h on 10 Sep, 32.34 h on 17 Sep; Haley Brown 28.50 h on 6 Sep (WO Hours from overlapping clocks).</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Working as intended — no ticket / We file TICKET-F2</t>
+          <t>— / We raise it (also check SV-10701)</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr"/>
@@ -3377,27 +4115,27 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>DQ-2</t>
+          <t>RQ-9</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Dashboard · Revenue (and the Sales report)</t>
+          <t>Export Reports · dates</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Should a work-order discount lower Revenue?</t>
+          <t>Should the export's dates use the location's own time zone?</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Today it does: $135.00 labor with a $20.00 discount counts as $115.00 (S1-38200). The PRD says "sum of invoice subtotals … before any discount", but the invoice's own Subtotal line is $115.00, so the sentence can be read both ways.</t>
+          <t>For Staging Heavy Duty - 9919 (time zone Asia/Karachi on staging) the Customer Invoice export prints dates one day earlier than the location's calendar date for invoices made late in the UTC day (e.g. S2-31625: 02 Sep in the file, 03 Sep at the location). Lethbridge (Edmonton) matches. Likely only a staging set-up artefact.</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Working as intended — no ticket (and the PRD wording could say "after work-order discounts") / We file TICKET-F4</t>
+          <t>— / —</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr"/>
@@ -3405,27 +4143,27 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>DQ-3</t>
+          <t>DQ-1</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Dashboard · Revenue split</t>
+          <t>Dashboard · Technician Efficiency (and the Technician Efficiency report)</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>When credits or discounts make a share negative, is "Parts -28% · Labor 130% · Other -2%" the intended display?</t>
+          <t>When a customer declines a line, should that line's technician time still count in "Invoiced Tech Hrs" (and its clocked time in "Clocked")?</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>It is arithmetically right (the three add to 100) but may confuse users</t>
+          <t>Today it does. Example S1-38198: only line 1 was billed, yet the technician shows 2.00 Invoiced Tech Hrs and 133.33 %. The Billing Efficiency tile leaves the same declined line out. The PRD calls the figure "invoiced technician hours" but defines it as "technician time *recorded* on work order lines".</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>— / Say how it should read</t>
+          <t>Working as intended — no ticket / We file TICKET-F2</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr"/>
@@ -3433,30 +4171,86 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
+          <t>DQ-2</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard · Revenue (and the Sales report)</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Should a work-order discount lower Revenue?</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Today it does: $135.00 labor with a $20.00 discount counts as $115.00 (S1-38200). The PRD says "sum of invoice subtotals … before any discount", but the invoice's own Subtotal line is $115.00, so the sentence can be read both ways.</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Working as intended — no ticket (and the PRD wording could say "after work-order discounts") / We file TICKET-F4</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>DQ-3</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard · Revenue split</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>When credits or discounts make a share negative, is "Parts -28% · Labor 130% · Other -2%" the intended display?</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>It is arithmetically right (the three add to 100) but may confuse users</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>— / Say how it should read</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
           <t>DQ-4</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Dashboard · Technician Utilization</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>The PRD says WO hours ÷ (WO + internal hours); the build divides by all clocked time. They agree today because no clock can be on neither. Confirm the PRD formula is the one to keep?</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>Latent difference</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="E44" s="3" t="inlineStr">
         <is>
           <t>— / —</t>
         </is>
       </c>
-      <c r="F42" s="3" t="inlineStr"/>
+      <c r="F44" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Dashboard + reports: screen-only filter, closed-ticket review, Chris question doc
- Left out 10 items a customer cannot reach on screen (QA lead rule).
- SV-8974 / SV-8927 safe to reopen; SV-8926 / SV-8930 not (spec stale / symptom fixed), asked PO.
- 39-question Chris Ward doc (Google Doc) in the established question-doc shape.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D95Q7VoyGzYXAt4w5J2bJE
</commit_message>
<xml_diff>
--- a/build/dashboard-verify-2026-10-28/ShopView-Dashboard-and-Reports-Full-Check-Findings-2026-10-28.xlsx
+++ b/build/dashboard-verify-2026-10-28/ShopView-Dashboard-and-Reports-Full-Check-Findings-2026-10-28.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Already reported" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="QA lead decision" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Not a ticket" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="PO questions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Questions for Chris" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Left out - not on screen" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -513,7 +514,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
@@ -564,7 +565,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
@@ -1245,7 +1246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1873,7 +1874,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>FU1</t>
+          <t>TE1</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1883,44 +1884,44 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Follow Up (hidden page)</t>
+          <t>Technician Efficiency</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>The hidden Follow Up page is blank and its data request fails (server error) on 12 of 12 reads.</t>
+          <t>A clock shorter than 0.01 h drops the line's whole technician time.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>12/12 reads HTTP 500.</t>
+          <t>727 rows, 221 lines.</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>No written source</t>
+          <t>see candidate</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>SQ-5</t>
+          <t>SQ-6</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>reports/W2-sales-advisor-tax/defects/TICKET-W2-5-follow-up-report-server-error.wiki</t>
+          <t>reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-te-tiny-clock-drops-tech-time.md</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/defects/TICKET-W2-5-follow-up-report-server-error.wiki</t>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-te-tiny-clock-drops-tech-time.md</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>TE1</t>
+          <t>DATE1</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1930,44 +1931,44 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Technician Efficiency</t>
+          <t>SBC / SBR date options</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>A clock shorter than 0.01 h drops the line's whole technician time.</t>
+          <t>The date options on screen match neither spec.</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>727 rows, 221 lines.</t>
+          <t>Screen.</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>see candidate</t>
+          <t>SBC v22 / SBR v30</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>SQ-6</t>
+          <t>SQ-7</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-te-tiny-clock-drops-tech-time.md</t>
+          <t>reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-date-filter-options.md</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-te-tiny-clock-drops-tech-time.md</t>
+          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-date-filter-options.md</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>DATE1</t>
+          <t>TAX2</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1977,82 +1978,35 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>SBC / SBR date options</t>
+          <t>Sales Tax Collected</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>The date options on screen match neither spec.</t>
+          <t>Unpaid invoices are not listed; credit-memo tax handling; $0.00 invoices listed "Paid" with no payment (643); deposit invoices dated by invoice not deposit (20).</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Screen.</t>
+          <t>See RESULTS §6.</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>SBC v22 / SBR v30</t>
+          <t>SV-4573</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>SQ-7</t>
+          <t>SQ-8, SQ-9, SQ-11</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-date-filter-options.md</t>
+          <t>reports/W2-sales-advisor-tax/RESULTS.md</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/defects/DEFECT-CANDIDATE-date-filter-options.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>TAX2</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Reports</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Sales Tax Collected</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Unpaid invoices are not listed; credit-memo tax handling; $0.00 invoices listed "Paid" with no payment (643); deposit invoices dated by invoice not deposit (20).</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>See RESULTS §6.</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>SV-4573</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>SQ-8, SQ-9, SQ-11</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>reports/W2-sales-advisor-tax/RESULTS.md</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/RESULTS.md</t>
         </is>
@@ -2606,12 +2560,12 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>SV-8927 (closed Obsolete)</t>
+          <t>SV-8927 (closed Obsolete). Spec v. 13 Aug still S3-R12/S3-R13/S8-R3 word for word; no later decision found</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Reopen?</t>
+          <t>Verdict: SAFE TO REOPEN</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -2653,12 +2607,12 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>SV-8926 (closed Obsolete)</t>
+          <t>SV-8926 (closed Obsolete). Spec still says "Total", but every other report screen says "Totals"</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Reopen?</t>
+          <t>Verdict: DO NOT REOPEN — asked Chris (doc Q20)</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -2700,12 +2654,12 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>SV-8930 (closed Obsolete)</t>
+          <t>SV-8930 (closed Obsolete). Original symptom (no message at all) is FIXED; only the words differ, and the suite now shows one shared message; precedent SV-9452</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Reopen?</t>
+          <t>Verdict: DO NOT REOPEN — asked Chris (doc Q21)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -2747,12 +2701,12 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>SV-8974 (closed OBSOLETE 9 Aug 2026 without a fix)</t>
+          <t>SV-8974 (closed OBSOLETE 9 Aug 2026 without a fix). SBR spec v30 (21 Oct) restates S6-R9 word for word</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Reopen?</t>
+          <t>Verdict: SAFE TO REOPEN</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -2777,7 +2731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2841,186 +2795,45 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>F3/F5</t>
+          <t>SBC2</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Billing Efficiency / Sales</t>
+          <t>Sales By Customer</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Lines added to Paid/Invoiced work orders after invoicing change hours and the pending invoice.</t>
+          <t>Asset label follows SV-9459, not spec S8-R7; SBC/SBR differ from today's Stats tab after later clocks or credits.</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Only possible through the API (no New Line button on screen) → Rule 24 pass; API-hardening note.</t>
+          <t>7,293 / 558 rows. Spec update (SQ-4) and design question (SQ-10).</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SBC v22, SV-9459</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SQ-4, SQ-10</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>defect-pack-2026-10-28/NOT-FILED.md</t>
+          <t>reports/W2-sales-advisor-tax/RESULTS.md</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/defect-pack-2026-10-28/NOT-FILED.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>W1-N1/N2</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Reports</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>WIP / Shop Efficiency</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Fixed price + hourly rate valued at hours × rate; void invoice hours counted.</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Only reachable through the API → Rule 24.</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>WQ-9</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>reports/W1-labor-wip/defects/NOT-FILED.md</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W1-labor-wip/defects/NOT-FILED.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>SBC2</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Reports</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Sales By Customer</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Asset label follows SV-9459, not spec S8-R7; SBC/SBR differ from today's Stats tab after later clocks or credits.</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>7,293 / 558 rows. Spec update (SQ-4) and design question (SQ-10).</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>SBC v22, SV-9459</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>SQ-4, SQ-10</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>reports/W2-sales-advisor-tax/RESULTS.md</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/RESULTS.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>O4-W2</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Outside reports</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Customer payment window</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Void invoice S1-38207 still shows $135.00 owing in New Customer Payment; work order stays "Invoiced".</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>The invoice was voided through the API only (no screen path) — passed to the payments owner as an observation.</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>reports/W2-sales-advisor-tax/RESULTS.md</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/claude/credit-memo-document-location-tov2x1/build/dashboard-verify-2026-10-28/reports/W2-sales-advisor-tax/RESULTS.md</t>
         </is>
@@ -3037,1220 +2850,1067 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>Doc #</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Project · feature</t>
+          <t>Our id</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Question</t>
+          <t>Question (report and point)</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Why we ask</t>
+          <t>Google Doc</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Outcomes</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
           <t>Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>DQ-1</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard, Technician Efficiency: a line the customer declined</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>DQ-2</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard, Revenue: a discount on the work order</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>DQ-3</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard, Revenue split when a share is negative</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>WQ-1</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Work In Progress, Days Open</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>WQ-3</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Work In Progress, how a negative amount is written</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>WQ-4</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Work In Progress, a part marked "received later"</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>WQ-5</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Work In Progress, an in-stock part not yet picked</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>WQ-11</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Work In Progress, an estimate with nothing approved</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>WQ-2</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Technician Utilization, decimal places</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>WQ-10</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Technician Utilization, a technician with only a few seconds clocked</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>WQ-8</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Technician Utilization and Timesheet Activities, time on a deleted work order</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>WQ-7</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Shop Efficiency, a shift that is still running</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>PQ-1</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Parts Velocity, how long "Last 90 days" is</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>PQ-2</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Parts Velocity, which date a sale is counted on</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>PQ-3</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Parts Velocity, a return to the vendor</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>PQ-4</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Parts Velocity, the Location column with one location picked</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>PQ-5</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Parts Velocity, the list of date options</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>PQ-7</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Parts Velocity, Last Sale for a sale with no stock movement</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>PQ-8</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Inventory Value, a cost above the highest price band</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>IQ-1</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Inventory Value, the words "Total" and "Qty"</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>IQ-2</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Inventory Value, the message when nothing matches</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>SQ-1</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Sales By Customer, what Margin % is divided by</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>SQ-2</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Sales By Customer and Sales By Representative, decimals and negative amounts</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>SQ-3</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Sales By Representative, a $0.00 invoice nobody paid</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>SQ-4</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Sales By Customer, the asset name</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>SQ-7</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Sales By Customer and Sales By Representative, the list of date options</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>SQ-10</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Sales By Customer and Sales By Representative, time clocked or parts credited after invoicing</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>SQ-6</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Technician Efficiency, a clock shorter than 36 seconds</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>SQ-8</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Sales Tax Collected, unpaid invoices</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>SQ-9</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Sales Tax Collected, tax on credit memos</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>SQ-11</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Sales Tax Collected, $0.00 invoices and deposit dates</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>RQ-1</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>A/R Aging Collection and A/P Aging Detail, a credit made on the chosen day</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>RQ-2</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>A/R Aging, a deposit on a part sale</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>RQ-3</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>IBS Batches, the total of a sent batch</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>RQ-5</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>IBS Batches, a $0.00 invoice</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>RQ-4</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Notes Report, more than 100 notes</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>RQ-6</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>QB Unexported, the No. column</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>RQ-7</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Export Reports, Terms on the Customer Invoice export</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>RQ-8</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Export Reports, more than 24 hours in a day on the Payroll Timesheet export</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1mEcB4cpsOqZXeim0vzmlbam2xSB02YshnyYRY0dk9s8/edit</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>What it was</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Why a customer cannot reach it</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>WQ-1</t>
+          <t>F3 / F5 (dashboard)</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Report Suite · Work In Progress</t>
+          <t>Lines added to a Paid / Invoiced work order change invoiced hours and a pending invoice</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Should "Days Open" count whole 24-hour periods (spec S4-R12), not calendar dates?</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Today it counts dates: S2-38105, created 28 Oct 3:19 PM, shows "1 days" ten hours later. The spec says elapsed time ÷ 24 h, floored ("a same-day work order shows 0 days"). The build's notes say dates were chosen to match the Work Orders list.</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>We file TICKET-W1-D1 / Keep as built; reword S4-R12 and §4</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr"/>
+          <t>No *New Line* button on a Paid or Invoiced work order — only the server API can do it</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>WQ-2</t>
+          <t>W1 N1</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Report Suite · Technician Utilization</t>
+          <t>WIP values a line with both an hourly rate and a fixed price at hours × rate</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Should Utilization % show one decimal place (spec S2-R7, e.g. 66.7%)?</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>It shows two (85.71%). SV-9059 (Done) asked for two; SV-9407 (same symptom as ours) was closed OBSOLETE with no comment; the spec still says one.</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>We file TICKET-W1-D2 / Keep two; update S2-R7</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr"/>
+          <t>The screen makes the two exclusive; set only through the API</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>WQ-3</t>
+          <t>W1 N2 / WQ-9</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Report Suite · Work In Progress (and the suite)</t>
+          <t>Shop Efficiency counts a void invoice's hours</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Should a negative amount read "-$3.13" (WIP spec S4-R14) rather than "(-$3.13)"?</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>The Totals row shows "(-$3.13)". The build applies a "suite-wide" brackets-and-minus rule said to come from Sales By Representative §3.</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>We capture a row picture and draft a ticket / Update S4-R14 / S4-E3 / S4-R23 examples</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr"/>
+          <t>An invoice can only be voided through the API</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>WQ-4</t>
+          <t>W2 O4</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Report Suite · Work In Progress</t>
+          <t>Void invoice S1-38207 still shows $135.00 owing in New Customer Payment</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Should a part request marked "received later" count as Parts Remaining (as built)?</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>The spec only defines "received" (Earned) and "ordered but not yet received" (Remaining).</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Working as built / Say where it belongs</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr"/>
+          <t>Same: voided through the API only</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>WQ-5</t>
+          <t>W2 FU1 / SQ-5</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Report Suite · Work In Progress</t>
+          <t>Hidden Follow Up page is blank, data request fails</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Should an in-stock part not yet picked count as Parts Remaining (as built)?</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Spec S4-R18 says "ordered but not yet received"; an in-stock part was never ordered.</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Working as built / Say where it belongs</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr"/>
+          <t>Not in the menu; reachable only by typing the address</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>WQ-6</t>
+          <t>W1 WQ-6</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Labor · Payroll Timesheet (hidden page)</t>
+          <t>Hidden Payroll Timesheet page is empty, data request fails</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Is the hidden Payroll Timesheet page (`/reports/payroll-timesheet`) still meant to work?</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>It is not in the menu, shows an empty page, and its data request fails (server error) for every date option except Today. No written source describes the page (SV-2071 describes the export).</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>We draft a ticket / Treat as retired (remove the route)</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr"/>
+          <t>Not in the menu; reachable only by typing the address</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>WQ-7</t>
+          <t>W3 PQ-6</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Performance · Shop Efficiency</t>
+          <t>Past sales of a deleted part disappear from Parts Velocity</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Should Total Clocked Hours include a shift that is still running (less than 24 h)?</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Shop Efficiency leaves every running clock out; Technician Utilization counts a running shift up to now (your 2026-10-22 rule on SV-11688).</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>We draft a ticket / Working as built</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr"/>
+          <t>A sold part cannot be deleted from the screen</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>WQ-8</t>
+          <t>DQ-4 (dashboard)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Labor · Technician Utilization / Timesheet Activities</t>
+          <t>Utilization divides by all clocked time instead of WO + internal</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Should time clocked on a work order that was later deleted still count as WO Hours?</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>5 such clocks at Heavy Duty this year count as WO Hours and show a blank Work Order in Timesheet Activities.</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Working as built / We draft a ticket</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr"/>
+          <t>No screen can create a clock that is neither on a work order nor a department, so the two formulas never differ</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>WQ-9</t>
+          <t>W4 RQ-9</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Performance · Shop Efficiency</t>
+          <t>Export dates one day early at Heavy Duty</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Confirm a void invoice must not count in Total Invoiced Hours?</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Today it does (seeded S1-38208), but only an API call can void an invoice, so no ticket.</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Noted (API-hardening only) / Working as built</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr"/>
+          <t>Staging set-up artefact (location time zone set to Asia/Karachi on staging)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>WQ-10</t>
+          <t>W2 O1 / O2</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Report Suite · Technician Utilization</t>
+          <t>Sales By Representative invoice request ignores paging; a hidden server tax total</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Should a technician whose only clocks are a few seconds long be listed with 0.00 hours?</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Rows like that show Utilization "—", which S2-R7 calls unreachable.</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Working as built / Hide such rows</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>WQ-11</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Report Suite · Work In Progress (spec text)</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Should S4-E1 / S2-R4 be reworded to match S3-R5 and your SV-9027 ruling (an Estimates row is valued at its unapproved lines)?</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>The two parts of the spec disagree; the build follows S3-R5 / SV-9027.</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Reword / Say which wording wins</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>SQ-1</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Reports · Sales By Customer · Margin %</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Should Sales By Customer's Margin % be Margin ÷ Subtotal (shop supplies included in the bottom number)?</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>The SBC spec (v22, S7-R11, Terminology) says *"Margin divided by the row's Subtotal … Margin % is profit measured against total sales."* The SBR spec (v30, §3, newer) says *"Sales By Customer computes Margin % from the same Margin base"* — Subtotal minus Shop Supplies. The build follows the SBR wording. Example: TestVT1, Heavy Duty, This month — Margin $21,960.81, Subtotal $28,569.41, shop supplies $2,050.98 → screen 82.81 %, SBC wording 76.87 %. Affects every row with shop supplies (counts in RESULTS.md).</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>We file `defects/TICKET-W2-1-sbc-margin-percent-base.wiki` and the SBR spec context note needs correcting / Working as intended — please update SBC S7-R11 / Terminology to "Margin ÷ (Subtotal − Shop Supplies)"</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>SQ-2</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Reports · Sales By Customer and Sales By Representative · number format</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Should Labor Delta show one decimal (+1.5) and SBC Margin % one decimal (64.7 %), as both specs say?</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>SBC S12-R2 and SBR S9-R2 say Labor Delta is *"rounded to one decimal"*; SBC S7-R11 says Margin % *"to one decimal"*. SV-9199 / SV-9200 (your tickets, Aug 12) repeat *"signed one-decimal format (+2.0 / -14.0 / 0.0)"*. But SV-9068 and SV-9069 (Done, Aug 10, "SV standard is 2") changed SBC to two decimals, and the build shows two decimals on SBC and SBR (+112.64, +1.00, 82.81 %). Also: SBR §3 says *"Negative dollar values use accounting-convention parentheses — `($1,234.56)`"*; the SBR screen shows a negative margin as (-$2.50), with both brackets and a minus sign.</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Ticket needed (one decimal; brackets without the minus sign) / Working as intended — please update S12-R2, S9-R2, S7-R11 to two decimals and the §3 negative-money example</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>SQ-3</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Reports · Sales By Representative · Status badge</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Should a $0.00 invoice that nobody paid show "Unpaid"?</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>SBR spec v30 §3: *"A zero-total invoice with no payment applied is unpaid and maps to Unpaid."* SV-9217 (QA defect, Done 26 Aug) made it read Paid (the invoice itself goes straight to Paid). The build follows SV-9217.</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Ticket needed / Working as intended — please change the §3 sentence</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>SQ-4</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Reports · Sales By Customer · asset label</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Is SV-9459's label ("Unit # - Year Make Model", VIN only as a fallback) the rule to keep?</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>The build follows SV-9459 (your ticket, Done 10 Sep). The SBC spec v22 still says *"The asset label is the vehicle's VIN"* then Unit, then plate (S8-R7 to S8-R10, Key Decisions).</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>No ticket — please update S8-R7…R10 / Ticket needed (VIN first)</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>SQ-5</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Reports · Follow Up (hidden)</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Is the hidden Follow Up report (/reports/sales-follow-up) still supported?</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>It is not in the menu, and every request fails with a server error (HTTP 500, all four locations, last 3/6/12 months); the screen is completely blank. No written source exists for it (searches in RESULTS.md).</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>We file a ticket (candidate drafted) / Remove the screen / route; no ticket</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>SQ-6</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Reports · Technician Efficiency (both tabs)</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>When a technician's clocks on a line add up to less than 36 seconds (0.01 h), should the line's tech time still be credited to them?</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>Today the line is listed with 0.00 Tech Hrs: the whole tech time of the line is dropped (e.g. Lethbridge S3-15255 "Recommend Axle 3 right tires": 30 min tech time, one technician clocked 12 s → 0.00 instead of 0.50). SV-5450 says tech time is *"allocated proportionally"* and *"Each technician receives a proportional share"*, but also *"must follow the existing behavior … No changes to the calculation logic"* — the existing behaviour has the 0.01-hour cut-off, which no document mentions.</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Ticket needed (credit the share; show Efficiency as "—") / Working as intended</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>SQ-7</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Reports · Sales By Customer and Sales By Representative · Date filter</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Which list of date options is right for these two reports?</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>SBC S2-R2: nine options in the order *Last 12 Months … Last Week*, "no option labeled Custom". SBR S2-R2: *Today, Yesterday, This Week, This Month, Last Month, This Year, Last Year, This Quarter, Last Quarter, Custom*. Both screens show *This week, Last week, This month, Last month, This quarter, Last quarter, This year, Last year, Last 12 months, Custom* (the suite filter bar). Each window itself is correct (location time zone, weeks start Sunday).</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>— / Say which list governs</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>SQ-8</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Reports · Sales Tax Collected</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Should unpaid ("Invoiced") invoices be listable on Sales Tax Collected?</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>The draft PRD (Confluence 50200592 v12) says *"Sales tax report for all invoices, Paid, Partially Paid and Unpaid"* and a status filter for *"Invoiced, paid or Partially paid"*. The newer CS training page (215941122, 15 Jan 2026) and SV-4233 (*"Should not show any invoices that are 'Invoiced', should only display 'PAID'"*) say paid only. The build shows Paid and Partially Paid only, dated by the latest payment.</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>Ticket needed / Working as intended (draft PRD outdated)</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>SQ-9</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Reports · Sales Tax Collected · All tax rates</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Should the tax-rate totals take off the tax on credit memos (returns) made in the same dates?</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>No document says. Today the screen's footer and the All tax rates tab add up the listed invoices only (checked: they match, 64 of 64 date ranges); credit memos never appear on this report. The server also works out a second, reduced tax total that no screen shows.</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>Ticket needed (show credit memo tax) / Working as intended</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>SQ-10</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Reports · Sales By Customer and Sales By Representative · Labor Delta, Labor Margin, Parts Margin</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>When time is clocked, or a cost changes, after an invoice is made, should these reports keep the figures from when the invoice was made?</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Neither spec says which moment counts. SBC: *"Labor Delta — Hours invoiced minus hours worked"*; SBR §3: *"hours worked = the technician clocked (timesheet) hours recorded against that work order"*, *"Labor Margin = Labor Invoiced − the shop's labor cost"*. On most invoices the reports match the work order's Stats tab exactly. They differ on 370 invoices for Labor Delta, 119 for Labor Margin and 69 for Parts Margin (of about 8,000). All of these are invoices where time was clocked, or parts were credited, after the invoice was made (mostly automated-test customer TestVT1). Example: S2-38022, report Labor Delta +1.00, Stats tab today 2.00 invoiced − 0.00 worked.</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Working as intended — please add "as at the time of invoicing" to both specs / Ticket needed (use today's clocked hours and costs)</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>SQ-11</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Reports · Sales Tax Collected · Invoice Status and Invoice Paid Date</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>(a) Should a $0.00 invoice with no payment be listed as "Paid", with a paid date? (b) When a deposit taken before invoicing pays part of an invoice, should Invoice Paid Date be the deposit's date?</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>(a) 643 $0.00 invoices are listed as Paid with a paid date (the invoice's creation time), but no payment exists. 428 of them read *unpaid* on their own record. This is the same question as SQ-3, for this report. (b) SV-4573: *"for partially paid invoices, show the date of the latest payment"*. On 20 deposit invoices the report shows the time the invoice was made, not the deposit date (e.g. P2-2445: deposit 21 Oct, report 22 Oct). *(Separate from this: the same deposit invoices show "Paid" instead of "Partially Paid". That one is clear from SV-4573 and is drafted as a ticket, `defects/TICKET-W2-6-sales-tax-status-deposit-paid.wiki`.)*</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>(a) Working as intended (b) Ticket needed / (a) Ticket needed (b) Working as intended — please note in the story that a deposit counts on the day it is applied</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>PQ-1</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Report Suite · Parts Velocity</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Should Last 90 days cover exactly 90 days (today and the 89 days before it)? *Yes / No*</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Today it covers 91 days: on 28 Oct it runs 30 Jul – 28 Oct. SV-11514 only says "The default range is Last 90 Days."</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>PQ-2</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Report Suite · Parts Velocity</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Should Revenue, Margin, Avg Cost, Avg Sell, Sold (WO), Sold (Parts Sale) and every Special Order figure be dated by the invoice date? *Yes / No*</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>The spec (Story 5, "Work-order date") dates them by the work order's end date, but work orders do not get an end date (it is empty on the paid work order S2-17193 we opened, and the build's own notes say it is never filled), so the report uses the invoice date. A "Yes" means the spec should be updated; a "No" means we need a different date.</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>PQ-3</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Report Suite · Parts Velocity</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Should a return to the vendor made from Parts → Returns count in Units Returned? *Yes / No*</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>It does today (we returned 1 unit of ZZAUTOTEST-PV1-10282011 to the vendor and Units Returned went from 0 to 1; cancelling it put it back to 0). The spec names only "a work-order part return or a parts-sale credit".</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="3" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>PQ-4</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Report Suite · Parts Velocity</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>When a user who has several locations picks one location, should the Location column be hidden? *Yes / No*</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>It is hidden today. The spec says both: S2-R12 "when a single location is in scope the column is hidden", and S3-R10 / Key Decisions "shown by default … regardless of how many locations are currently selected". (This is the same open point as the contested SV-8938.) Inventory Value shows the column with one location selected.</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>PQ-5</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Report Suite · Parts Velocity</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Is the date list on screen the intended one — This week, Last week, This month, Last month, This quarter, Last quarter, This year, Last year, Last 90 days, Last 12 months, Custom (no Today, no Yesterday)? *Yes / No*</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>That is what the screen offers, in line with your 5 Aug answer and SV-11514. The spec text (S2-R2) still lists Today and Yesterday and does not list Last 12 months, so a "Yes" means S2-R2 should be updated. Every option's dates were checked and are right.</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr"/>
-      <c r="F28" s="3" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>PQ-6</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Report Suite · Parts Velocity</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Should a part's past sales stay in Parts Velocity after the part record is deleted? *Yes / No*</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>Today they disappear. Last Year at Staging Heavy Duty - 9919 is missing $2,357.74 of billed sales across 9 parts that no longer exist (for example 84-4005PK, billed on S2-4699, S2-4987, S2-6540). S3-N1 says "A part with billed Revenue &gt; 0 is always kept". We could not delete a sold part from the screen, so we have not raised a ticket.</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>PQ-7</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Report Suite · Parts Velocity</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Should Last Sale for a stocked part include a sale that was billed but recorded no stock movement? *Yes / No*</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>Example: N000000001069 at Staging Heavy Duty - 9919 was billed on S2-16621 (30 Jul 2026) but Last Sale reads 160 days (its previous stock-moving sale). S3-N1 calls a billed sale without stock movement "a drop-ship sale"; Last Sale is "the part's most recent sale".</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="3" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>PQ-8</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Report Suite · Inventory Value</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>When a part's cost is above the highest price band of its category's pricing matrix, should Unit Sell use that highest band's markup? *Yes / No*</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>That is what it does today, and it matches the parts list (example: 2599273C92 at Staging Lethbridge - 4310, cost $526.70, category HD-Filters whose bands stop at $500 → Unit Sell $752.44 = +42.86%). The spec only says "the shop's pricing-matrix markup on cost for that part's category".</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>RQ-1</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>A/R Aging Collection (and A/P Aging Detail) · Past Due</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Should a credit created ON the chosen date count as 0 days old — so it is left off A/R Aging Collection (and shows Past Due 0 on A/P Aging Detail)?</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>The PRD says "If the calculated days are ≤ 0 … it's not shown on the report". Ticket SV-5606 (Done, Jan 2026) asked instead for "Today's Credits … displayed with 1 as a Past Due", and the build does that. Example: CM2-4462 (E2E Credits Customer) created 30 Sep 2026 is listed as 1 day past due on 30 Sep 2026.</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>We file TICKET-AR1 / Working as intended — the PRD wording should be updated to match SV-5606</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>RQ-2</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>A/R Aging · part-sale deposits</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Should a deposit taken on a part sale reduce that part sale's open balance on A/R Aging once the part sale is invoiced (as it already does on the customer's Invoices tab)?</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>P2-2352 (TestVT1): Invoices tab $443.43, A/R Aging $543.43 — the $100 deposit DEP-4763 stays "Held" and A/R now leaves held deposits out (SV-11690 fix). Same for P2-2439 ($5).</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>We add this to SV-11690 (comment), or file it on your say-so / Working as intended</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>RQ-3</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>IBS Batches · Sent tab</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>Must a Sent batch's Total always equal the sum of the invoices (and credits) inside it?</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>Lethbridge batch of 2 Oct 2026 shows $9,473.35; its 9 invoices add up to $9,183.29 (its own IBS export also says $9,183.29). We could not find the cause.</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>We file TICKET-IBS1 and a developer finds the cause / —</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>RQ-4</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>Notes Report</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Should the Notes Report let the user see every note in the chosen range (today it stops at 100)?</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>"All" shows 100 of 2,545 notes; "Last Week" 100 of 255; "Filter by Author" 100 of 1,105. There is no "load more". No written spec exists for this report.</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>We file TICKET-NOTES1 / Working as intended (the 100 limit should then be stated on screen)</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>RQ-5</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>IBS Batches · Ready to Send</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>Should a $0.00 invoice be listed in Ready to Send?</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>S2-16924 (Fort Mohave Diesel Repair) is listed with Total $0.00 / Balance $0.00, waiting to be sent to IBS.</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>— / We raise it</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>RQ-6</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>QB Unexported · Customers tab</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Should every credit memo row show its credit number (e.g. CM2-4476) in the No. column?</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>All 283 credit-memo rows (Heavy Duty 255, Lethbridge 28) have a blank No.; payments / applications are blank too. 111 documents appear twice with two different errors. No written spec exists for this screen.</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>We raise it / —</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>RQ-7</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>Export Reports · Customer Invoice</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>Should the Terms column show the invoice's own term?</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>7 invoices from Sep 2026 show "Net 30/50/60" while the invoice and its customer both say COD and the due date equals the invoice date (e.g. S2-31597).</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>We raise it / —</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>RQ-8</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Export Reports · Payroll Timesheet</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>Can an employee's day legitimately exceed 24 Total Hours?</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>Sep 2026: Admin Shopview 40.70 h on 10 Sep, 32.34 h on 17 Sep; Haley Brown 28.50 h on 6 Sep (WO Hours from overlapping clocks).</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>— / We raise it (also check SV-10701)</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>RQ-9</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Export Reports · dates</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>Should the export's dates use the location's own time zone?</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>For Staging Heavy Duty - 9919 (time zone Asia/Karachi on staging) the Customer Invoice export prints dates one day earlier than the location's calendar date for invoices made late in the UTC day (e.g. S2-31625: 02 Sep in the file, 03 Sep at the location). Lethbridge (Edmonton) matches. Likely only a staging set-up artefact.</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>— / —</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>DQ-1</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>Dashboard · Technician Efficiency (and the Technician Efficiency report)</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>When a customer declines a line, should that line's technician time still count in "Invoiced Tech Hrs" (and its clocked time in "Clocked")?</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>Today it does. Example S1-38198: only line 1 was billed, yet the technician shows 2.00 Invoiced Tech Hrs and 133.33 %. The Billing Efficiency tile leaves the same declined line out. The PRD calls the figure "invoiced technician hours" but defines it as "technician time *recorded* on work order lines".</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>Working as intended — no ticket / We file TICKET-F2</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>DQ-2</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>Dashboard · Revenue (and the Sales report)</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>Should a work-order discount lower Revenue?</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>Today it does: $135.00 labor with a $20.00 discount counts as $115.00 (S1-38200). The PRD says "sum of invoice subtotals … before any discount", but the invoice's own Subtotal line is $115.00, so the sentence can be read both ways.</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>Working as intended — no ticket (and the PRD wording could say "after work-order discounts") / We file TICKET-F4</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>DQ-3</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>Dashboard · Revenue split</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>When credits or discounts make a share negative, is "Parts -28% · Labor 130% · Other -2%" the intended display?</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>It is arithmetically right (the three add to 100) but may confuse users</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>— / Say how it should read</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>DQ-4</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>Dashboard · Technician Utilization</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>The PRD says WO hours ÷ (WO + internal hours); the build divides by all clocked time. They agree today because no clock can be on neither. Confirm the PRD formula is the one to keep?</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>Latent difference</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>— / —</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr"/>
+          <t>Not visible on any screen</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Chris question doc v2: Section 1 Dashboard / Section 2 Reports, neutral wording, build and location per question
Rewritten in place in the same Google Doc (Docs batchUpdate; text verified byte-equal, 0 equations).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D95Q7VoyGzYXAt4w5J2bJE
</commit_message>
<xml_diff>
--- a/build/dashboard-verify-2026-10-28/ShopView-Dashboard-and-Reports-Full-Check-Findings-2026-10-28.xlsx
+++ b/build/dashboard-verify-2026-10-28/ShopView-Dashboard-and-Reports-Full-Check-Findings-2026-10-28.xlsx
@@ -2898,7 +2898,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Dashboard, Technician Efficiency: a line the customer declined</t>
+          <t>Dashboard · Technician Efficiency: a line the customer declined</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Dashboard, Revenue: a discount on the work order</t>
+          <t>Dashboard · Revenue: a discount on the work order</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Dashboard, Revenue split when a share is negative</t>
+          <t>Dashboard · Revenue split when a share is negative</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -2961,7 +2961,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Work In Progress, Days Open</t>
+          <t>Reports · Work In Progress: Days Open</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Work In Progress, how a negative amount is written</t>
+          <t>Reports · Work In Progress: how a negative amount is written</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -3003,7 +3003,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Work In Progress, a part marked "received later"</t>
+          <t>Reports · Work In Progress: a part marked "received later"</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Work In Progress, an in-stock part not yet picked</t>
+          <t>Reports · Work In Progress: an in-stock part not yet picked</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Work In Progress, an estimate with nothing approved</t>
+          <t>Reports · Work In Progress: an estimate with nothing approved</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Technician Utilization, decimal places</t>
+          <t>Reports · Technician Utilization: decimal places</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Technician Utilization, a technician with only a few seconds clocked</t>
+          <t>Reports · Technician Utilization: a technician with only a few seconds clocked</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Technician Utilization and Timesheet Activities, time on a deleted work order</t>
+          <t>Reports · Technician Utilization and Timesheet Activities: time on a deleted work order</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Shop Efficiency, a shift that is still running</t>
+          <t>Reports · Shop Efficiency: a shift that is still running</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -3150,7 +3150,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Parts Velocity, how long "Last 90 days" is</t>
+          <t>Reports · Parts Velocity: how long "Last 90 days" is</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -3171,7 +3171,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Parts Velocity, which date a sale is counted on</t>
+          <t>Reports · Parts Velocity: which date a sale is counted on</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Parts Velocity, a return to the vendor</t>
+          <t>Reports · Parts Velocity: a return to the vendor</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Parts Velocity, the Location column with one location picked</t>
+          <t>Reports · Parts Velocity: the Location column with one location picked</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Parts Velocity, the list of date options</t>
+          <t>Reports · Parts Velocity: the list of date options</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -3255,7 +3255,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Parts Velocity, Last Sale for a sale with no stock movement</t>
+          <t>Reports · Parts Velocity: Last Sale for a sale with no stock movement</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -3276,7 +3276,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Inventory Value, a cost above the highest price band</t>
+          <t>Reports · Inventory Value: a cost above the highest price band</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Inventory Value, the words "Total" and "Qty"</t>
+          <t>Reports · Inventory Value: the words "Total" and "Qty"</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Inventory Value, the message when nothing matches</t>
+          <t>Reports · Inventory Value: the message when nothing matches</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Sales By Customer, what Margin % is divided by</t>
+          <t>Reports · Sales By Customer: what Margin % is divided by</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Sales By Customer and Sales By Representative, decimals and negative amounts</t>
+          <t>Reports · Sales By Customer and Sales By Representative: decimals and negative amounts</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -3381,7 +3381,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Sales By Representative, a $0.00 invoice nobody paid</t>
+          <t>Reports · Sales By Representative: a $0.00 invoice nobody paid</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Sales By Customer, the asset name</t>
+          <t>Reports · Sales By Customer: the asset name</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Sales By Customer and Sales By Representative, the list of date options</t>
+          <t>Reports · Sales By Customer and Sales By Representative: the list of date options</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Sales By Customer and Sales By Representative, time clocked or parts credited after invoicing</t>
+          <t>Reports · Sales By Customer and Sales By Representative: time clocked or parts credited after invoicing</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Technician Efficiency, a clock shorter than 36 seconds</t>
+          <t>Reports · Technician Efficiency: a clock shorter than 36 seconds</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Sales Tax Collected, unpaid invoices</t>
+          <t>Reports · Sales Tax Collected: unpaid invoices</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Sales Tax Collected, tax on credit memos</t>
+          <t>Reports · Sales Tax Collected: tax on credit memos</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -3528,7 +3528,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Sales Tax Collected, $0.00 invoices and deposit dates</t>
+          <t>Reports · Sales Tax Collected: $0.00 invoices and deposit dates</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -3549,7 +3549,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>A/R Aging Collection and A/P Aging Detail, a credit made on the chosen day</t>
+          <t>Reports · A/R Aging Collection: a credit made on the chosen day</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>A/R Aging, a deposit on a part sale</t>
+          <t>Reports · A/R Aging: a deposit on a part sale</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -3591,7 +3591,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>IBS Batches, the total of a sent batch</t>
+          <t>Reports · IBS Batches: the total of a sent batch</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>IBS Batches, a $0.00 invoice</t>
+          <t>Reports · IBS Batches: a $0.00 invoice</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Notes Report, more than 100 notes</t>
+          <t>Reports · Notes Report: more than 100 notes</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>QB Unexported, the No. column</t>
+          <t>Reports · QB Unexported: the No. column</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Export Reports, Terms on the Customer Invoice export</t>
+          <t>Reports · Export Reports: Terms on the Customer Invoice export</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Export Reports, more than 24 hours in a day on the Payroll Timesheet export</t>
+          <t>Reports · Export Reports: more than 24 hours in a day on the Payroll Timesheet export</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">

</xml_diff>